<commit_message>
hw(bom): actualizar lista de componentes en PDF y CSV
</commit_message>
<xml_diff>
--- a/hardware/BOM-ASRS.xlsx
+++ b/hardware/BOM-ASRS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\SE-2026-ASRS\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD87BF8E-7ED7-4F81-BAF3-E7510604E5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0247F16F-E3E9-4EFD-9B16-F751EF67FA4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
     <t>RF-01 a RF-13, RNF-04, RNF-05</t>
   </si>
   <si>
-    <t>Incluye USB-Serial (CP2102). No requiere módulo externo para UART.</t>
+    <t>Incluye USB-Serial integrado.</t>
   </si>
   <si>
     <t>Capacitor bypass</t>
@@ -73,7 +73,7 @@
     <t>RNF-02</t>
   </si>
   <si>
-    <t>Desacoplo en riel 3.3V y 5V, lo más cerca posible del ESP32.</t>
+    <t>Bypass de alimentación del ESP32.</t>
   </si>
   <si>
     <t>Actuadores y drivers</t>
@@ -88,7 +88,7 @@
     <t>RF-01, RF-02</t>
   </si>
   <si>
-    <t>Eje vertical (levanta carro + producto). Torque ×5 sobre mínimo requerido.</t>
+    <t>Eje Y (vertical).</t>
   </si>
   <si>
     <t>Stepper NEMA17 — eje X</t>
@@ -97,7 +97,7 @@
     <t>17HS2408, 0.6 A, 16 N·cm</t>
   </si>
   <si>
-    <t>Eje horizontal. Carga mínima, motor más pequeño reduce consumo.</t>
+    <t>Eje X (horizontal).</t>
   </si>
   <si>
     <t>Driver DRV8825</t>
@@ -109,7 +109,7 @@
     <t>RF-01, RF-02, RF-10</t>
   </si>
   <si>
-    <t>Microstepping 1/32. Pin ENABLE compartido conectado al E-Stop por hardware.</t>
+    <t>Microstepping 1/32. ENABLE conectado al E-Stop.</t>
   </si>
   <si>
     <t>Servo MG996R</t>
@@ -121,7 +121,7 @@
     <t>RF-03, RF-04, RF-05</t>
   </si>
   <si>
-    <t>Extractor del end-effector. Control PWM a 50 Hz, 1 pin GPIO.</t>
+    <t>Extractor del end-effector. PWM 50 Hz.</t>
   </si>
   <si>
     <t>Capacitor electrolítico</t>
@@ -130,7 +130,7 @@
     <t>100 µF 25V (uno por driver)</t>
   </si>
   <si>
-    <t>OBLIGATORIO en cada DRV8825. Sin estos los drivers se dañan con picos de corriente.</t>
+    <t>Uno por driver. Obligatorio para proteger el DRV8825.</t>
   </si>
   <si>
     <t>Sensores</t>
@@ -145,7 +145,7 @@
     <t>RF-06, RF-07</t>
   </si>
   <si>
-    <t>Rango útil 10–1000 g. Montada en el end-effector. 4 hilos: E+, E–, A+, A–.</t>
+    <t>Rango 10–1000 g. Montada en el end-effector.</t>
   </si>
   <si>
     <t>Op-amp LM358N</t>
@@ -154,7 +154,7 @@
     <t>Dual op-amp, DIP-8, single supply 3–32V</t>
   </si>
   <si>
-    <t>3 ICs: IC1 (buffers E1), IC2 (diferenciador E1 + filtro E2), IC3 (amp. final E3). Alimentar a 5V.</t>
+    <t>IC1: buffers, IC2: diferenciador + filtro, IC3: amp. final.</t>
   </si>
   <si>
     <t>Resistencia Rg</t>
@@ -166,7 +166,7 @@
     <t>RF-06</t>
   </si>
   <si>
-    <t>Etapa 1 — fija ganancia diferencial G₁=21×. Nodo central a GND.</t>
+    <t>Ganancia G₁=21×.</t>
   </si>
   <si>
     <t>Resistencias red OA3</t>
@@ -175,7 +175,7 @@
     <t>10 kΩ · 1% · 1/4W</t>
   </si>
   <si>
-    <t>Etapa 1 — R1, R2, R3, R4 alrededor del diferenciador OA3. 1% mismo lote para máximo CMRR.</t>
+    <t>Red resistiva OA3. Usar 1% mismo lote.</t>
   </si>
   <si>
     <t>Resistencias divisor Vref</t>
@@ -184,7 +184,7 @@
     <t>10 kΩ · 5% · 1/4W</t>
   </si>
   <si>
-    <t>Etapa 1 — Rdiv1 y Rdiv2. Generan Vref=2.5V (5V÷2). Bypass con 100nF.</t>
+    <t>Divisor Vref=2.5V.</t>
   </si>
   <si>
     <t>Resistencias filtro Sallen-Key</t>
@@ -193,13 +193,13 @@
     <t>160 kΩ · 5% · 1/4W</t>
   </si>
   <si>
-    <t>Etapa 2 — R5 y R6. Con C=100nF → fc=9.95 Hz. Rechaza ruido steppers y 50 Hz.</t>
+    <t>Filtro Sallen-Key, fc≈10 Hz.</t>
   </si>
   <si>
     <t>Resistencia Rin amp. final</t>
   </si>
   <si>
-    <t>Etapa 3 — resistencia de entrada OA5. Con Rf=47kΩ → G₃=5.7×.</t>
+    <t>Entrada OA5, G₃=5.7×.</t>
   </si>
   <si>
     <t>Resistencia Rf amp. final</t>
@@ -208,7 +208,7 @@
     <t>47 kΩ · 1% · 1/4W</t>
   </si>
   <si>
-    <t>Etapa 3 — resistencia de retroalimentación OA5. G₃ = 1 + 47k/10k = 5.7×.</t>
+    <t>Retroalimentación OA5.</t>
   </si>
   <si>
     <t>Capacitores 100 nF C0G</t>
@@ -217,7 +217,7 @@
     <t>100 nF · C0G · 25V</t>
   </si>
   <si>
-    <t>Bypass VCC IC1/IC2/IC3 (×3), bypass Vref (×1), filtro Sallen-Key C4 y C5 (×2), reserva (×2).</t>
+    <t>Bypass VCC (×3), Vref (×1), filtro Sallen-Key (×2), reserva (×2).</t>
   </si>
   <si>
     <t>Expansor I/O MCP23017</t>
@@ -229,7 +229,7 @@
     <t>RF-03, RF-04, RF-07, RF-09, RNF-04</t>
   </si>
   <si>
-    <t>I2C addr 0x20 (A0=A1=A2=GND). 16 GPIO: 12 para microswitches + 4 disponibles. Pull-ups 4.7kΩ en SDA/SCL si es DIP.</t>
+    <t>I2C addr 0x20. 12 GPIO para microswitches. Pull-ups 4.7kΩ en SDA/SCL si es DIP.</t>
   </si>
   <si>
     <t>Microswitch mini</t>
@@ -241,7 +241,7 @@
     <t>RF-03, RF-04, RF-07, RF-09</t>
   </si>
   <si>
-    <t>Uno por celda (3×4=12). Detectan presencia de producto. Terminal NC a GND, COM al CD74HC4067.</t>
+    <t>Uno por celda (3×4=12). NC a GND, COM al MCP23017.</t>
   </si>
   <si>
     <t>Sensor IR TCRT5000</t>
@@ -253,7 +253,7 @@
     <t>RF-07</t>
   </si>
   <si>
-    <t>Presencia en end-effector. Validación cruzada con celda de carga.</t>
+    <t>Presencia en end-effector.</t>
   </si>
   <si>
     <t>Endstop mecánico con PCB</t>
@@ -265,7 +265,7 @@
     <t>RF-01, RF-11</t>
   </si>
   <si>
-    <t>2 por eje (homing + límite). Usan pull-up interno del ESP32.</t>
+    <t>2 por eje: homing y límite.</t>
   </si>
   <si>
     <t>Alimentación</t>
@@ -277,7 +277,7 @@
     <t>60W, conector barrel jack</t>
   </si>
   <si>
-    <t>Alimenta DRV8825 y entrada del DC-DC. NO usar fuente de laboratorio.</t>
+    <t>Alimenta DRV8825 y módulo DC-DC.</t>
   </si>
   <si>
     <t>Módulo DC-DC LM2596</t>
@@ -286,7 +286,7 @@
     <t>Buck ajustable, 12V → 5V, 3A</t>
   </si>
   <si>
-    <t>Alimenta ESP32, servo, sensores y circuito acondicionamiento. Ajustar a 5.0V antes de conectar.</t>
+    <t>Genera riel 5V. Ajustar a 5.0V antes de conectar cargas.</t>
   </si>
   <si>
     <t>Transformador 24V AC</t>
@@ -295,7 +295,7 @@
     <t>220V AC → 24V AC, 5VA mínimo</t>
   </si>
   <si>
-    <t>Alimenta las 3 luces piloto a través de los relés. 5VA suficiente para 3 luces.</t>
+    <t>Alimentación 24V AC para luces piloto.</t>
   </si>
   <si>
     <t>Conector barrel jack hembra</t>
@@ -304,7 +304,7 @@
     <t>5.5×2.1 mm, panel mount</t>
   </si>
   <si>
-    <t>Entrada de alimentación principal a la carcasa.</t>
+    <t>Entrada de alimentación 12V.</t>
   </si>
   <si>
     <t>Seguridad</t>
@@ -319,7 +319,7 @@
     <t>RF-10</t>
   </si>
   <si>
-    <t>Corta ENABLE de ambos DRV8825 por hardware, sin pasar por firmware.</t>
+    <t>Corta ENABLE de los DRV8825 por hardware.</t>
   </si>
   <si>
     <t>Indicadores</t>
@@ -334,7 +334,7 @@
     <t>RF-12</t>
   </si>
   <si>
-    <t>Estado sistema: operativo (verde), advertencia (amarillo), error/fault (rojo).</t>
+    <t>Verde: operativo, amarillo: advertencia, rojo: error.</t>
   </si>
   <si>
     <t>Relé 5V</t>
@@ -343,7 +343,7 @@
     <t>5V bobina, contacto 250V AC 10A</t>
   </si>
   <si>
-    <t>Uno por luz piloto. Bobina controlada por transistor BC547 desde GPIO ESP32.</t>
+    <t>Uno por luz piloto. Controlado por BC547.</t>
   </si>
   <si>
     <t>Transistor BC547</t>
@@ -352,7 +352,7 @@
     <t>NPN, TO-92</t>
   </si>
   <si>
-    <t>Driver de la bobina del relé. Base via resistencia 1kΩ desde GPIO 3.3V del ESP32.</t>
+    <t>Driver del relé desde GPIO ESP32.</t>
   </si>
   <si>
     <t>Diodo 1N4007</t>
@@ -361,7 +361,7 @@
     <t>Rectificador, 1A 1000V</t>
   </si>
   <si>
-    <t>Flyback en paralelo con la bobina del relé. Protege el transistor de picos inductivos.</t>
+    <t>Protección flyback en la bobina del relé.</t>
   </si>
   <si>
     <t>Resistencia base transistor</t>
@@ -370,7 +370,7 @@
     <t>1 kΩ · 5% · 1/4W</t>
   </si>
   <si>
-    <t>Limita corriente de base del BC547. Una por transistor.</t>
+    <t>Limitadora de base del BC547.</t>
   </si>
   <si>
     <t>Tarjeta y componentes pasivos</t>
@@ -385,7 +385,7 @@
     <t>RNF-03</t>
   </si>
   <si>
-    <t>Principal (MCU + drivers) y auxiliar si se requiere.</t>
+    <t>Tarjeta principal y auxiliar.</t>
   </si>
   <si>
     <t>Tarjeta perforada pequeña</t>
@@ -394,7 +394,7 @@
     <t>3×5 cm, doble cara</t>
   </si>
   <si>
-    <t>PCB del preamp (Etapa 1) en el end-effector. IC1 + Rg + conectores.</t>
+    <t>Preamp en el end-effector.</t>
   </si>
   <si>
     <t>Estaño 60/40</t>
@@ -403,7 +403,7 @@
     <t>0.8 mm, rollo</t>
   </si>
   <si>
-    <t>Soldadura de la tarjeta.</t>
+    <t>Soldadura.</t>
   </si>
 </sst>
 </file>

</xml_diff>